<commit_message>
Replace Netflix citation suggestion with verified search-specific articles
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VtPXTbweeL2ybNtP3anhQX
</commit_message>
<xml_diff>
--- a/AI_NAS影视音乐搜索评估_竞品对照评审.xlsx
+++ b/AI_NAS影视音乐搜索评估_竞品对照评审.xlsx
@@ -1931,7 +1931,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="165" customHeight="1">
+    <row r="21" ht="320" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>附录</t>
@@ -1959,12 +1959,14 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>更贴切的替换案例：Netflix 搜索的拼写容错与稀疏 query 处理（Netflix TechBlog 搜索相关文章）；Amazon Prime Video X-Ray（演员/角色场景识别，佐证演员搜索与长期多模态方向）；TMDB/Trakt API 文档（元数据与归属数据来源）；QNAP Qsirch / Synology Universal Search（NAS 直接竞品的搜索能力基线）。</t>
+          <t>建议替换为 Netflix 搜索方向的直接资料（均已核实可访问）：
+【消费端搜索】① Lamkhede &amp; Das《Challenges in Search on Streaming Services: Netflix Case Study》SIGIR 2019（arxiv.org/abs/1903.04638，即时搜索/多语言/库外查询，对应§2/§11）；② 《Search Personalization at Netflix》WWW 2023（dl.acm.org/doi/10.1145/3543873.3587675，排序个性化，对应§10/§13）；③ 《Recommendations and Results Organization in Netflix Search》RecSys 2021（dl.acm.org/doi/10.1145/3460231.3474602，结果组织与空结果处理，对应§10 降级策略）；④ Netflix 2025-05 上线 OpenAI 驱动的自然语言『vibe』搜索（techcrunch.com/2025/05/07/netflix-debuts-its-generative-ai-powered-search-tool，对应§2/§6 主观偏好词的消费端形态）。
+【TechBlog 工程侧】⑤ 《The AI Evolution of Graph Search at Netflix》（netflixtechblog.com/the-ai-evolution-of-graph-search-at-netflix-d416ec5b1151，LLM 将自然语言转结构化 filter，直接对应§10/§13 槽位抽取）；⑥ 《Global Languages Support at Netflix: Testing Search Queries》（netflixtechblog.com/global-languages-support-at-netflix-testing-search-queries-ede40f7d93d3，多语言搜索质量测试，对应§11）；⑦ 《Building In-Video Search》与《Powering Multimodal Intelligence for Video Search》（netflixtechblog.com/building-in-video-search-936766f0017c，片段/多模态检索，注意是内部剪辑工具场景，对应§1/§14 长期方向）。另补：Prime Video X-Ray、TMDB/Trakt API、QNAP Qsirch / Synology Universal Search（NAS 能力基线）。</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>替换两条推荐系统引用为上述搜索类直接案例；补充 NAS 直接竞品（Qsirch/Universal Search）作为能力基线对标，让评估依据与『NAS 上的搜索』场景完全对齐。</t>
+          <t>替换两条推荐系统引用为上述搜索类直接案例（按消费端/工程侧分组、标注对应章节）；引用⑦时注明其为 Netflix 内部制作侧工具而非消费端搜索，避免评审误读；补充 NAS 直接竞品（Qsirch/Universal Search）作为能力基线对标。</t>
         </is>
       </c>
     </row>
@@ -2344,17 +2346,17 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>microgenres 细分标签体系（Cerebral 等数千主观标签）；搜索拼写容错与稀疏 query 处理</t>
+          <t>microgenres 细分标签体系（Cerebral 等数千主观标签）；搜索方向公开资料充足：SIGIR 2019 案例研究（即时搜索/多语言/库外查询）、RecSys 2021 结果组织、WWW 2023 搜索个性化、TechBlog《The AI Evolution of Graph Search》（LLM→结构化 filter）、《Global Languages Support: Testing Search Queries》；2025-05 消费端上线 OpenAI 驱动自然语言『vibe』搜索</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>支持：主观标签可体系化运营；提示：文档附录引用的是其推荐系统资料而非搜索资料，应替换</t>
+          <t>支持：主观标签可体系化运营；『自然语言→结构化条件』的技术路线与文档§13 同构；提示：文档附录引用的是其推荐系统资料而非上述搜索资料，应替换（具体清单见影视评审明细·附录行）</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>影视§6/附录</t>
+          <t>影视§2/§6/§13/附录</t>
         </is>
       </c>
     </row>

</xml_diff>